<commit_message>
Add brand prefix to hwahae-verified names
</commit_message>
<xml_diff>
--- a/output/discovery10shops_with_hwahae.xlsx
+++ b/output/discovery10shops_with_hwahae.xlsx
@@ -436,7 +436,7 @@
     <col width="45" customWidth="1" min="2" max="2"/>
     <col width="40" customWidth="1" min="3" max="3"/>
     <col width="45" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -484,7 +484,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>톤업 뽀용 크림 [01 화이트]</t>
+          <t>AOU 톤업 뽀용 크림 [01 화이트]</t>
         </is>
       </c>
     </row>
@@ -511,7 +511,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>심콩 샴푸 [호텔우드]</t>
+          <t>헤트라스 심콩 샴푸 [호텔우드]</t>
         </is>
       </c>
     </row>
@@ -538,7 +538,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>시크릿 모공 세라마이드 버블 오일 에센스 미스트</t>
+          <t>숨37 시크릿 모공 세라마이드 버블 오일 에센스 미스트</t>
         </is>
       </c>
     </row>
@@ -565,7 +565,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>오리진 퓨어 밸런싱 클렌징 오일</t>
+          <t>ATRUE 오리진 퓨어 밸런싱 클렌징 오일</t>
         </is>
       </c>
     </row>
@@ -592,7 +592,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>워터 캡슐 선세럼  [SPF50+</t>
+          <t>리쥬란 워터 캡슐 선세럼  [SPF50+</t>
         </is>
       </c>
     </row>
@@ -619,7 +619,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>포어 타이트닝 클렌징밤</t>
+          <t>리쥬란 포어 타이트닝 클렌징밤</t>
         </is>
       </c>
     </row>
@@ -673,7 +673,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>살롱10 프로페셔널 시카프로틴 샴푸</t>
+          <t>미장센 살롱10 프로페셔널 시카프로틴 샴푸</t>
         </is>
       </c>
     </row>
@@ -700,7 +700,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>그린토마토 NMN 포어 리프팅 앰플</t>
+          <t>성분에디터 그린토마토 그린토마토 NMN 포어 리프팅 앰플</t>
         </is>
       </c>
     </row>
@@ -722,7 +722,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>링클바운스 멀티밤</t>
+          <t>가히 링클바운스 멀티밤</t>
         </is>
       </c>
     </row>
@@ -749,7 +749,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>녹두 약산성 클렌징폼</t>
+          <t>비플레인 녹두 약산성 클렌징폼</t>
         </is>
       </c>
     </row>
@@ -776,7 +776,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>프로바이오덤 3D 리프팅크림</t>
+          <t>바이오힐보 프로바이오덤 3D 리프팅크림</t>
         </is>
       </c>
     </row>
@@ -803,7 +803,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>DW EGF 세럼 (디더블유이지에프세럼)</t>
+          <t>이지듀 DW EGF 세럼 (디더블유이지에프세럼)</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>그로우턴 엑소좀 브러쉬 앰플</t>
+          <t>릴리이브 그로우턴 엑소좀 브러쉬 앰플</t>
         </is>
       </c>
     </row>
@@ -857,7 +857,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>인리치 본딩 케어 샴푸</t>
+          <t>아윤채 인리치 본딩 케어 샴푸</t>
         </is>
       </c>
     </row>
@@ -884,7 +884,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>아토베리어365 캡슐 토너</t>
+          <t>에스트라 아토베리어365 캡슐 토너</t>
         </is>
       </c>
     </row>
@@ -911,7 +911,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>리프레싱 클렌징 폼</t>
+          <t>헤라 리프레싱 클렌징 폼</t>
         </is>
       </c>
     </row>
@@ -938,7 +938,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>판테놀 리퀴드 에센스 선세럼 [SPF50+</t>
+          <t>달바 판테놀 리퀴드 에센스 선세럼 [SPF50+</t>
         </is>
       </c>
     </row>
@@ -965,7 +965,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>글로우업 인샤워 톤업밀크</t>
+          <t>메디픽미 글로우업 인샤워 톤업밀크</t>
         </is>
       </c>
     </row>
@@ -992,7 +992,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>(해외) 리피 펜슬 [미 어게인]</t>
+          <t>AGAIN ME (해외) 리피 펜슬 [미 어게인]</t>
         </is>
       </c>
     </row>
@@ -1019,7 +1019,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>엠지에프 리턴 크림</t>
+          <t>셀메딕스 엠지에프 리턴 크림</t>
         </is>
       </c>
     </row>
@@ -1046,7 +1046,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>짱구 에디션 아크네 클리어 퍼퓸 바디워시</t>
+          <t>포먼트 짱구 에디션 아크네 클리어 퍼퓸 바디워시</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1100,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>티트리 시카 포어 코팩</t>
+          <t>브링그린 티트리 시카 포어 코팩</t>
         </is>
       </c>
     </row>
@@ -1122,7 +1122,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>워터풀 선크림 [SPF50+</t>
+          <t>달바 워터풀 선크림 [SPF50+</t>
         </is>
       </c>
     </row>
@@ -1144,7 +1144,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>레티날 샷 타이트닝 부스터</t>
+          <t>셀리맥스 레티날 샷 타이트닝 부스터</t>
         </is>
       </c>
     </row>
@@ -1171,7 +1171,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>피디알엔 리들샷 나이트 크림</t>
+          <t>VT코스메틱 피디알엔 리들샷 나이트 크림</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add volume to hwahae-verified names, also cleaned up truncated bracket artifacts (e.g. trailing [SPF50+)
</commit_message>
<xml_diff>
--- a/output/discovery10shops_with_hwahae.xlsx
+++ b/output/discovery10shops_with_hwahae.xlsx
@@ -484,7 +484,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>AOU 톤업 뽀용 크림 [01 화이트]</t>
+          <t>AOU 톤업 뽀용 크림 [01 화이트] 100ml</t>
         </is>
       </c>
     </row>
@@ -511,7 +511,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>헤트라스 심콩 샴푸 [호텔우드]</t>
+          <t>헤트라스 심콩 샴푸 [호텔우드] 1013ml</t>
         </is>
       </c>
     </row>
@@ -538,7 +538,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>숨37 시크릿 모공 세라마이드 버블 오일 에센스 미스트</t>
+          <t>숨37 시크릿 모공 세라마이드 버블 오일 에센스 미스트 60ml</t>
         </is>
       </c>
     </row>
@@ -565,7 +565,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>ATRUE 오리진 퓨어 밸런싱 클렌징 오일</t>
+          <t>ATRUE 오리진 퓨어 밸런싱 클렌징 오일 150ml</t>
         </is>
       </c>
     </row>
@@ -592,7 +592,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>리쥬란 워터 캡슐 선세럼  [SPF50+</t>
+          <t>리쥬란 워터 캡슐 선세럼 40ml×2개</t>
         </is>
       </c>
     </row>
@@ -619,7 +619,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>리쥬란 포어 타이트닝 클렌징밤</t>
+          <t>리쥬란 포어 타이트닝 클렌징밤 50ml×2개</t>
         </is>
       </c>
     </row>
@@ -673,7 +673,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>미장센 살롱10 프로페셔널 시카프로틴 샴푸</t>
+          <t>미장센 살롱10 프로페셔널 시카프로틴 샴푸 480ml×2개</t>
         </is>
       </c>
     </row>
@@ -700,7 +700,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>성분에디터 그린토마토 그린토마토 NMN 포어 리프팅 앰플</t>
+          <t>성분에디터 그린토마토 그린토마토 NMN 포어 리프팅 앰플 40ml+40ml</t>
         </is>
       </c>
     </row>
@@ -722,7 +722,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>가히 링클바운스 멀티밤</t>
+          <t>가히 링클바운스 멀티밤 3개입</t>
         </is>
       </c>
     </row>
@@ -749,7 +749,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>비플레인 녹두 약산성 클렌징폼</t>
+          <t>비플레인 녹두 약산성 클렌징폼 160ml</t>
         </is>
       </c>
     </row>
@@ -776,7 +776,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>바이오힐보 프로바이오덤 3D 리프팅크림</t>
+          <t>바이오힐보 프로바이오덤 3D 리프팅크림 50ml</t>
         </is>
       </c>
     </row>
@@ -803,7 +803,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>이지듀 DW EGF 세럼 (디더블유이지에프세럼)</t>
+          <t>이지듀 DW EGF 세럼 (디더블유이지에프세럼) 2개</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>릴리이브 그로우턴 엑소좀 브러쉬 앰플</t>
+          <t>릴리이브 그로우턴 엑소좀 브러쉬 앰플 130ml</t>
         </is>
       </c>
     </row>
@@ -857,7 +857,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>아윤채 인리치 본딩 케어 샴푸</t>
+          <t>아윤채 인리치 본딩 케어 샴푸 350g</t>
         </is>
       </c>
     </row>
@@ -884,7 +884,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>에스트라 아토베리어365 캡슐 토너</t>
+          <t>에스트라 아토베리어365 캡슐 토너 300ml</t>
         </is>
       </c>
     </row>
@@ -911,7 +911,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>헤라 리프레싱 클렌징 폼</t>
+          <t>헤라 리프레싱 클렌징 폼 50g</t>
         </is>
       </c>
     </row>
@@ -938,7 +938,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>달바 판테놀 리퀴드 에센스 선세럼 [SPF50+</t>
+          <t>달바 판테놀 리퀴드 에센스 선세럼 50ml</t>
         </is>
       </c>
     </row>
@@ -965,7 +965,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>메디픽미 글로우업 인샤워 톤업밀크</t>
+          <t>메디픽미 글로우업 인샤워 톤업밀크 300g</t>
         </is>
       </c>
     </row>
@@ -992,7 +992,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>AGAIN ME (해외) 리피 펜슬 [미 어게인]</t>
+          <t>AGAIN ME (해외) 리피 펜슬 [미 어게인] 400ml</t>
         </is>
       </c>
     </row>
@@ -1019,7 +1019,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>셀메딕스 엠지에프 리턴 크림</t>
+          <t>셀메딕스 엠지에프 리턴 크림 70ml</t>
         </is>
       </c>
     </row>
@@ -1046,7 +1046,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>포먼트 짱구 에디션 아크네 클리어 퍼퓸 바디워시</t>
+          <t>포먼트 짱구 에디션 아크네 클리어 퍼퓸 바디워시 500ml</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1100,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>브링그린 티트리 시카 포어 코팩</t>
+          <t>브링그린 티트리 시카 포어 코팩 5매입</t>
         </is>
       </c>
     </row>
@@ -1122,7 +1122,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>달바 워터풀 선크림 [SPF50+</t>
+          <t>달바 워터풀 선크림</t>
         </is>
       </c>
     </row>
@@ -1144,7 +1144,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>셀리맥스 레티날 샷 타이트닝 부스터</t>
+          <t>셀리맥스 레티날 샷 타이트닝 부스터 15ml</t>
         </is>
       </c>
     </row>

</xml_diff>